<commit_message>
Finalize Research 1.0 public release
</commit_message>
<xml_diff>
--- a/audit/audit_log.xlsx
+++ b/audit/audit_log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/limingda/Desktop/research1.0/audit/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07D5DCEB-62B8-CF40-8D9A-FA15DEE70122}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD8BC75D-D86C-9442-B4BD-2B2828B0CA8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="720" windowWidth="29400" windowHeight="18400" xr2:uid="{6FDB4A4A-A627-EE4C-A970-1AAED24F5C63}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="163">
   <si>
     <t>date</t>
   </si>
@@ -498,6 +498,33 @@
   </si>
   <si>
     <t>The Q29–Qwen score correction changed several aggregate and reliability results. The final analysis and documentation were updated so that all reported results are consistent with the corrected scored_responses.csv.</t>
+  </si>
+  <si>
+    <t>Re-ran the final analysis after the Q29–Qwen correction and updated the Notebook and README to reflect the corrected descriptive, inferential, and inter-rater reliability results</t>
+  </si>
+  <si>
+    <t>public_data_packaging</t>
+  </si>
+  <si>
+    <t>The analysis notebook depended on local research files containing raw model responses and other non-public evaluation material</t>
+  </si>
+  <si>
+    <t>Created public_analysis_scores.csv and public_second_rater_scores.csv containing only the fields needed to reproduce the quantitative and inter-rater reliability analyses</t>
+  </si>
+  <si>
+    <t>To improve reproducibility while keeping raw model responses and other non-public evaluation material out of the public analysis files</t>
+  </si>
+  <si>
+    <t>final_validation</t>
+  </si>
+  <si>
+    <t>Final public-facing files had not yet undergone a complete post-packaging consistency and methodological documentation check</t>
+  </si>
+  <si>
+    <t>Completed final validation of the public-safe datasets, notebook reproducibility, methodological limitations, evaluation documentation, and qualitative case-study release safety</t>
+  </si>
+  <si>
+    <t>Final review confirmed that the public analysis files contain 120 main responses and 32 second-rater responses with no missing values or duplicate question-model pairs, reproduced the final reported results, and aligned the public-facing documentation with the final evaluation methodology and release restrictions. No additional scoring changes were made.</t>
   </si>
 </sst>
 </file>
@@ -552,7 +579,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -562,6 +589,9 @@
     </xf>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -877,7 +907,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA39CE57-C41E-F74F-9A55-C244D7D0F100}">
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:G47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="1"/>
@@ -886,7 +916,7 @@
     <col min="4" max="4" width="10.83203125" style="1"/>
     <col min="5" max="5" width="33.1640625" style="1" customWidth="1"/>
     <col min="6" max="6" width="27.5" style="1" customWidth="1"/>
-    <col min="7" max="7" width="39" style="1" customWidth="1"/>
+    <col min="7" max="7" width="45" style="1" customWidth="1"/>
     <col min="8" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
@@ -1902,7 +1932,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="45" spans="1:7" ht="102" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:7" ht="119" x14ac:dyDescent="0.2">
       <c r="A45" s="3">
         <v>46274</v>
       </c>
@@ -1919,10 +1949,56 @@
         <v>152</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="G45" s="1" t="s">
         <v>153</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" ht="136" x14ac:dyDescent="0.2">
+      <c r="A46" s="3">
+        <v>46277</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E46" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="F46" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="G46" s="1" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" ht="153" x14ac:dyDescent="0.2">
+      <c r="A47" s="3">
+        <v>46277</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E47" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="F47" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="G47" s="1" t="s">
+        <v>162</v>
       </c>
     </row>
   </sheetData>

</xml_diff>